<commit_message>
Update internal networking page data and reconciliation logic
</commit_message>
<xml_diff>
--- a/assets/Strategy & Operations Service Lines.xlsx
+++ b/assets/Strategy & Operations Service Lines.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://impactadvisors3-my.sharepoint.com/personal/martin_you_impact-advisors_com/Documents/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://impactadvisors3-my.sharepoint.com/personal/martin_you_impact-advisors_com/Documents/Desktop/Internal Networking Page VS Code/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3A49A3C7-4F9F-4959-85D2-6CD16742BA05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="8_{3A49A3C7-4F9F-4959-85D2-6CD16742BA05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D17FA383-7424-4CDA-A601-0DE276EA8CD0}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{AAB7EEAF-11CB-4475-B2F2-A15F99F765BD}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="859" uniqueCount="490">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="865" uniqueCount="494">
   <si>
     <t>Name</t>
   </si>
@@ -1574,6 +1574,18 @@
   </si>
   <si>
     <t>Holly.ezell@impact-advisors.com</t>
+  </si>
+  <si>
+    <t>Anya Mehta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Labor </t>
+  </si>
+  <si>
+    <t>Anya Mehta | LinkedIn</t>
+  </si>
+  <si>
+    <t>anya.mehta@impact-advisors.com</t>
   </si>
 </sst>
 </file>
@@ -1675,8 +1687,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8700CBAD-FC9E-4C75-BB7D-18040C7D2A47}" name="Table1" displayName="Table1" ref="A1:F140" totalsRowShown="0">
-  <autoFilter ref="A1:F140" xr:uid="{8700CBAD-FC9E-4C75-BB7D-18040C7D2A47}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8700CBAD-FC9E-4C75-BB7D-18040C7D2A47}" name="Table1" displayName="Table1" ref="A1:F141" totalsRowShown="0">
+  <autoFilter ref="A1:F141" xr:uid="{8700CBAD-FC9E-4C75-BB7D-18040C7D2A47}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{B7225A69-4070-43CE-AFA1-930CE8ABA093}" name="Name"/>
     <tableColumn id="2" xr3:uid="{74BF9A37-C28E-424C-A808-B2BBA42CFA48}" name="Service Line"/>
@@ -2055,7 +2067,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09DBBB96-A9E5-4CC1-B781-70890184EE77}">
-  <dimension ref="A1:I140"/>
+  <dimension ref="A1:I141"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21.453125" bestFit="1" customWidth="1"/>
@@ -4876,6 +4888,26 @@
       </c>
       <c r="F140" s="1" t="s">
         <v>489</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A141" t="s">
+        <v>490</v>
+      </c>
+      <c r="B141" t="s">
+        <v>491</v>
+      </c>
+      <c r="C141" t="s">
+        <v>442</v>
+      </c>
+      <c r="D141" t="s">
+        <v>9</v>
+      </c>
+      <c r="E141" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="F141" s="1" t="s">
+        <v>493</v>
       </c>
     </row>
   </sheetData>
@@ -5027,10 +5059,12 @@
     <hyperlink ref="E139" r:id="rId145" display="https://www.linkedin.com/in/liam-ford-6075b1213/" xr:uid="{15B31879-B400-48DE-A3F9-1BF55BC45271}"/>
     <hyperlink ref="E140" r:id="rId146" xr:uid="{EA224624-EE80-4FC0-8A49-F7F1CA6414B2}"/>
     <hyperlink ref="F140" r:id="rId147" xr:uid="{0692CBCB-6A78-42AD-A3D0-B5B9DE759520}"/>
+    <hyperlink ref="E141" r:id="rId148" display="Holly Ezell | LinkedIn" xr:uid="{EC9F1A40-858A-411C-8FF6-DC5E3C533A99}"/>
+    <hyperlink ref="F141" r:id="rId149" xr:uid="{2C7806E6-EB85-450E-8BF3-A3907B57728E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId148"/>
+    <tablePart r:id="rId150"/>
   </tableParts>
 </worksheet>
 </file>
@@ -5153,6 +5187,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010062AC75732FCC574AA39F1F73CAC12435" ma:contentTypeVersion="7" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="63221f8ce7b9bdba850c731f1f8526dd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="18c801aa-b08e-4147-8d71-4a4146fc5f82" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a6e5fe67e0597052bb7d02be10438d84" ns2:_="">
     <xsd:import namespace="18c801aa-b08e-4147-8d71-4a4146fc5f82"/>
@@ -5314,12 +5354,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -5330,6 +5364,22 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CFA9E554-1ADE-46CE-8803-AC258E13C25F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="18c801aa-b08e-4147-8d71-4a4146fc5f82"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{887352FC-8020-462A-8C14-3CDA6EDFB226}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5347,22 +5397,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CFA9E554-1ADE-46CE-8803-AC258E13C25F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="18c801aa-b08e-4147-8d71-4a4146fc5f82"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{898626DD-6B53-4F3D-BC27-4B5A8D32B3B3}">
   <ds:schemaRefs>

</xml_diff>